<commit_message>
data: publish 2026-10-09 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-09-182路.xlsx
+++ b/data/export/2026-10-09-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,17 +693,17 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -709,13 +713,17 @@
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>1/12</t>
         </is>
       </c>
     </row>
@@ -776,7 +784,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -815,7 +823,7 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
@@ -826,7 +834,7 @@
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -887,7 +895,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -926,7 +934,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -937,7 +945,7 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -965,32 +973,36 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>79分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -998,7 +1010,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1022,17 +1034,17 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -1042,13 +1054,17 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB5" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>79.0</t>
+        </is>
+      </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>2/12</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1125,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1159,7 +1175,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1236,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1286,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1347,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1397,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1405,22 @@
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>沪A68870D</t>
+          <t>沪A55712D</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>07:28</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1437,12 +1453,12 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1456,7 +1472,7 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -1492,7 +1508,673 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-09 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-09-182路.xlsx
+++ b/data/export/2026-10-09-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC28"/>
+  <dimension ref="A1:AC33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>8/13</t>
+          <t>11/13</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -948,12 +948,12 @@
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>92.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>10/13</t>
+          <t>8/13</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1057,22 +1057,22 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>81.0</t>
+          <t>84.5</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>7/13</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1176,22 +1176,22 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA6" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>85.0</t>
+          <t>83.5</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>4/13</t>
+          <t>5/13</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>6/13</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1419,17 +1419,17 @@
       </c>
       <c r="AA8" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>5/13</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA9" s="2" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>5/13</t>
+          <t>9/13</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>5/13</t>
+          <t>9/13</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1776,17 +1776,17 @@
       </c>
       <c r="AA11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>91.0</t>
+          <t>79.5</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>8/13</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>12/13</t>
+          <t>13/13</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>10/13</t>
+          <t>12/13</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>8/13</t>
+          <t>11/13</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr">
@@ -2296,24 +2296,24 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>09:47</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>92分钟</t>
+          <t>87分钟</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2372,12 +2372,12 @@
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>92.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>10/13</t>
+          <t>8/13</t>
         </is>
       </c>
     </row>
@@ -2405,32 +2405,36 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>88分钟</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -2438,7 +2442,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2462,37 +2466,37 @@
       </c>
       <c r="W17" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA17" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>81.0</t>
+          <t>84.5</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>7/13</t>
         </is>
       </c>
     </row>
@@ -2520,32 +2524,36 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>81分钟</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
           <t>07:52</t>
@@ -2553,7 +2561,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2577,33 +2585,37 @@
       </c>
       <c r="W18" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y18" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA18" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>—/13</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -2631,32 +2643,36 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>82分钟</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -2664,7 +2680,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2688,37 +2704,37 @@
       </c>
       <c r="W19" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA19" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
-          <t>85.0</t>
+          <t>83.5</t>
         </is>
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>4/13</t>
+          <t>5/13</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2795,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2833,7 +2849,7 @@
       </c>
       <c r="AC20" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>6/13</t>
         </is>
       </c>
     </row>
@@ -2861,32 +2877,36 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -2894,7 +2914,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2918,17 +2938,17 @@
       </c>
       <c r="W21" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z21" s="2" t="inlineStr">
@@ -2938,17 +2958,17 @@
       </c>
       <c r="AA21" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>5/13</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3029,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3048,7 +3068,7 @@
       </c>
       <c r="Z22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA22" s="2" t="inlineStr">
@@ -3063,7 +3083,7 @@
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>5/13</t>
+          <t>9/13</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3144,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3178,7 +3198,7 @@
       </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>5/13</t>
+          <t>9/13</t>
         </is>
       </c>
     </row>
@@ -3206,32 +3226,36 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -3239,7 +3263,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3263,17 +3287,17 @@
       </c>
       <c r="W24" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z24" s="2" t="inlineStr">
@@ -3283,17 +3307,17 @@
       </c>
       <c r="AA24" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
-          <t>91.0</t>
+          <t>79.5</t>
         </is>
       </c>
       <c r="AC24" s="2" t="inlineStr">
         <is>
-          <t>8/13</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3378,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3408,7 +3432,7 @@
       </c>
       <c r="AC25" s="2" t="inlineStr">
         <is>
-          <t>12/13</t>
+          <t>13/13</t>
         </is>
       </c>
     </row>
@@ -3469,7 +3493,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3523,7 +3547,7 @@
       </c>
       <c r="AC26" s="2" t="inlineStr">
         <is>
-          <t>10/13</t>
+          <t>12/13</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3608,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3638,7 +3662,7 @@
       </c>
       <c r="AC27" s="2" t="inlineStr">
         <is>
-          <t>8/13</t>
+          <t>11/13</t>
         </is>
       </c>
     </row>
@@ -3646,22 +3670,22 @@
       <c r="A28" s="2" t="inlineStr"/>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>沪A67026D</t>
+          <t>沪A13735A</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
           <t>川沙客运站</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>金杨路金口路</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3699,7 +3723,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3713,47 +3737,622 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr">
         <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB28" s="2" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="AC28" s="2" t="inlineStr">
+        <is>
+          <t>1/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
           <t>10:15</t>
         </is>
       </c>
-      <c r="V28" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W28" s="2" t="inlineStr">
+      <c r="W29" s="2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X28" s="2" t="inlineStr">
-        <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="Y28" s="2" t="inlineStr">
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="Z28" s="2" t="inlineStr">
+      <c r="Z29" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA28" s="2" t="inlineStr">
+      <c r="AA29" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB28" s="2" t="inlineStr">
-        <is>
-          <t>92.0</t>
-        </is>
-      </c>
-      <c r="AC28" s="2" t="inlineStr">
-        <is>
-          <t>10/13</t>
+      <c r="AB29" s="2" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>8/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB30" s="2" t="inlineStr">
+        <is>
+          <t>84.5</t>
+        </is>
+      </c>
+      <c r="AC30" s="2" t="inlineStr">
+        <is>
+          <t>7/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>沪A08953A</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
+      <c r="AC31" s="2" t="inlineStr">
+        <is>
+          <t>3/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr"/>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="inlineStr"/>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB32" s="2" t="inlineStr">
+        <is>
+          <t>83.5</t>
+        </is>
+      </c>
+      <c r="AC32" s="2" t="inlineStr">
+        <is>
+          <t>5/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y33" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB33" s="2" t="inlineStr">
+        <is>
+          <t>90.0</t>
+        </is>
+      </c>
+      <c r="AC33" s="2" t="inlineStr">
+        <is>
+          <t>9/13</t>
         </is>
       </c>
     </row>

</xml_diff>